<commit_message>
chore(audit): blog editorial audit results for posts 21-25
Tracker updated with 4-layer audit (fact check / AI slop / quality /
tone) for:
- 21 best-mtb-trails-belfast (8/10, fixed)
- 22 best-mtb-trails-ireland (8/10, passed)
- 23 best-mtb-trails-wicklow (7/10, FLAGGED)
- 24 best-online-cycling-coach-how-to-choose (9/10, fixed)
- 25 best-road-cycling-routes-ireland (7/10, FLAGGED)

Two posts flagged for human review on factual concerns: Wicklow article
recommends riding boardwalks on the Wicklow Way (walker infrastructure)
and references unverified bike shop name; Ireland routes article makes
a specific claim about Ring of Kerry tour bus direction that conflicts
with established convention.

Code edits committed separately on branch claude/epic-heyrovsky-0329c7.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/blog-audit-tracker.xlsx
+++ b/blog-audit-tracker.xlsx
@@ -1598,42 +1598,40 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REVIEWED — FIXED</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PASS (minor: Rostrevor distance inconsistency 30km vs 40km, fixed)</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>8</v>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Anthony voice; direct, Irish references, peer-to-peer; no fluff</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Internal distance inconsistency at Rostrevor (30km in body/FAQ vs 40km in trail box)</t>
         </is>
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Unified trail box to 30km to match body, FAQ, excerpt, answerCapsule</t>
         </is>
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Editorial Auditor (Opus 4.7)</t>
         </is>
       </c>
     </row>
@@ -1648,42 +1646,40 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REVIEWED — PASSED</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PASS (15 trail centres verified: Ballinastoe, Ticknock, Glencullen, Carrick, Ballyhoura, Killaloe, Killarney NP, Gap of Dunloe, Coolaney, Derroura, Portumna, Rostrevor, Carlingford, Davagh, Castlewellan)</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>LOW (a few "world-class"/"hidden gem" repeats but in moderation)</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>8</v>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>On-voice Anthony; "quick-hit list" close is excellent; Coillte/Forest Service NI accuracy good</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>None significant</t>
         </is>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>None — committed as-is</t>
         </is>
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Editorial Auditor (Opus 4.7)</t>
         </is>
       </c>
     </row>
@@ -1698,42 +1694,40 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>FLAGGED — NEEDS REVIEW</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ISSUES: (1) Ballinastoe described with green/blue/red/black graded loops — Coillte officially lists blue/red/black; "green" attribution questionable. (2) Recommends riding Djouce boardwalks on the Wicklow Way — boardwalks are walker infrastructure on a National Waymarked Way; goes against trail-access etiquette the article itself preaches. (3) "Trailriders in Roundwood" bike shop name unverified.</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>LOW (voice is mostly clean: "ice rinks", "bread and butter" are voicey)</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>7</v>
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Voice OK; closing line strong; seasonal breakdown solid</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Trail-grading attribution at Ballinastoe needs verification; Wicklow Way boardwalk recommendation needs reconsideration; bike shop name needs verification</t>
         </is>
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>None — flagged for human review per audit rules (quality 7 = flag only)</t>
         </is>
       </c>
       <c r="J24" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Editorial Auditor (Opus 4.7)</t>
         </is>
       </c>
     </row>
@@ -1748,42 +1742,40 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REVIEWED — FIXED</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PASS (NDY athlete results match brand bible Cat 3→Cat 1 reference; 1,400 episodes plausible; pricing range plausible for online coaching)</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>LOW (sharp, voice-matched: "managing a spreadsheet", "set of power files rather than a human being")</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>9</v>
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Strong on-voice: anti-list-bait opener "I am not going to give you a ranked list"; casual authority drops; FTP-obsession callout matches Anthony</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pricing "150-300 per month" missing currency</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Added euro symbols: €150-€300/month (consistent with brand bible coaching package range €175-€1,250)</t>
         </is>
       </c>
       <c r="J25" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Editorial Auditor (Opus 4.7)</t>
         </is>
       </c>
     </row>
@@ -1798,42 +1790,40 @@
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>FLAGGED — NEEDS REVIEW</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>POSSIBLE ERROR: Ring of Kerry — article says "tourist buses run clockwise, do anti-clockwise to avoid them". Tour buses on Ring of Kerry traditionally run ANTI-CLOCKWISE per long-standing tour-operator convention; cyclists are typically advised to ride clockwise to face buses or anti-clockwise WITH bus traffic. The articles claim about bus direction needs verification. All other route facts (Conor Pass 456m, Healy Pass, Slea Head 47km, Inishowen, Mournes, Kilmacthomas viaduct ~30m) check out.</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>MEDIUM — answerCapsule uses "blow your mind" (off-voice per voice guide which forbids hype like "you wont believe"). "stunning"/"world-class" used several times. Em-dashes inconsistent: this post uses "--" while posts 21-24 use "—".</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>7</v>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Body voice mostly OK; "savour rather than suffer", "hammer" are voicey. answerCapsule is hyped/salesy — off-brand.</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ring of Kerry bus direction claim; answerCapsule hype phrases; "--" formatting throughout (vs "—" elsewhere); duplicated FAQ section at bottom of body</t>
         </is>
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>None — flagged for human review per audit rules (quality 7 = flag only)</t>
         </is>
       </c>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Editorial Auditor (Opus 4.7)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(audit): blog editorial audit results for posts 16-20, 26-45
Tracker updated with 6-axis quality scores (voice match, slop kill list,
cycling specificity, narrative quality, structural clarity, SEO integration)
for the next 25 unswept posts. All 25 now at or above the 9.5/10 editorial
standard: 1 PASS (biggest-training-mistakes-from-coaches), 24 FIXED via
surgical edits committed in five separate content commits on this branch.

Pending count: 209 → 184.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/blog-audit-tracker.xlsx
+++ b/blog-audit-tracker.xlsx
@@ -94,7 +94,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -126,6 +126,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFE2FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -177,7 +182,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -256,6 +261,18 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1346,44 +1363,44 @@
           <t>best-cycling-podcast-for-triathletes</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J17" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H17" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I17" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1396,44 +1413,44 @@
           <t>best-cycling-podcasts-2026</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E18" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="inlineStr">
+        <is>
+          <t>genuinely x2; italic emphasis</t>
+        </is>
+      </c>
+      <c r="I18" s="28" t="inlineStr">
+        <is>
+          <t>Stripped genuinely; removed italics</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1446,44 +1463,44 @@
           <t>best-cycling-training-podcasts-age-groupers</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J19" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E19" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F19" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H19" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I19" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1496,44 +1513,44 @@
           <t>best-gravel-trails-ireland</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E20" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="inlineStr">
+        <is>
+          <t>genuinely x3; world-class; stunning; NDY</t>
+        </is>
+      </c>
+      <c r="I20" s="28" t="inlineStr">
+        <is>
+          <t>Stripped slop; reframed claims; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1546,44 +1563,44 @@
           <t>best-indoor-cycling-podcasts-winter</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E21" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I21" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1836,44 +1853,44 @@
           <t>best-roadman-episodes-masters</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="inlineStr">
+        <is>
+          <t>soft closer; missing article; NDY</t>
+        </is>
+      </c>
+      <c r="I27" s="28" t="inlineStr">
+        <is>
+          <t>Tightened closer; added article; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J27" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1886,44 +1903,44 @@
           <t>best-roadman-episodes-nutrition</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C28" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H28" s="28" t="inlineStr">
+        <is>
+          <t>limp opener; NDY abbreviation</t>
+        </is>
+      </c>
+      <c r="I28" s="28" t="inlineStr">
+        <is>
+          <t>Sharpened opener; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J28" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1936,44 +1953,44 @@
           <t>best-roadman-episodes-time-crunched</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C29" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D29" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E29" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F29" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H29" s="28" t="inlineStr">
+        <is>
+          <t>opener voice</t>
+        </is>
+      </c>
+      <c r="I29" s="28" t="inlineStr">
+        <is>
+          <t>Added Anthony opener pattern</t>
+        </is>
+      </c>
+      <c r="J29" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1986,44 +2003,44 @@
           <t>biggest-training-mistakes-from-coaches</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F30" s="30" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G30" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H30" s="30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I30" s="30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J30" s="30" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2036,44 +2053,44 @@
           <t>bike-fit-one-change-amateurs-should-make</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D31" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E31" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F31" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H31" s="28" t="inlineStr">
+        <is>
+          <t>changes everything; key takeaways soup; weak opener; NDY</t>
+        </is>
+      </c>
+      <c r="I31" s="28" t="inlineStr">
+        <is>
+          <t>Rewrote opener, body, ending into prose; killed bullet soup; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J31" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2086,44 +2103,44 @@
           <t>bike-leg-of-triathlon-why-age-groupers-get-it-wrong</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D32" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F32" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I32" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J32" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E32" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F32" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H32" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I32" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J32" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2136,44 +2153,44 @@
           <t>breathing-techniques-cycling-performance</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E33" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F33" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="inlineStr">
+        <is>
+          <t>straightforward; accountability pillar; in order to; absolute; genuinely; NDY</t>
+        </is>
+      </c>
+      <c r="I33" s="28" t="inlineStr">
+        <is>
+          <t>Stripped slop; replaced accountability→community; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J33" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2186,44 +2203,44 @@
           <t>brick-workouts-for-ironman</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C34" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E34" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F34" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H34" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I34" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J34" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2236,44 +2253,44 @@
           <t>carbohydrate-per-hour-cyclists</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E35" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F35" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H35" s="28" t="inlineStr">
+        <is>
+          <t>genuinely x2; NDY expansion</t>
+        </is>
+      </c>
+      <c r="I35" s="28" t="inlineStr">
+        <is>
+          <t>Stripped genuinely; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J35" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2286,44 +2303,44 @@
           <t>comeback-cyclist-12-week-return-plan</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E36" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I36" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J36" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E36" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F36" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H36" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I36" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J36" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2336,44 +2353,44 @@
           <t>common-training-mistakes-from-1400-podcast-episodes</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D37" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E37" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F37" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H37" s="28" t="inlineStr">
+        <is>
+          <t>genuinely x5; flat opener</t>
+        </is>
+      </c>
+      <c r="I37" s="28" t="inlineStr">
+        <is>
+          <t>Stripped genuinely; tightened opener with 1,400+ framing</t>
+        </is>
+      </c>
+      <c r="J37" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2386,44 +2403,44 @@
           <t>courtney-conley-cycling-shoes-fit</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G38" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H38" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I38" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J38" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C38" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E38" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F38" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G38" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H38" s="28" t="inlineStr">
+        <is>
+          <t>episode number in prose; highest-leverage; flat opener</t>
+        </is>
+      </c>
+      <c r="I38" s="28" t="inlineStr">
+        <is>
+          <t>Stripped ep-2107; replaced highest-leverage; sharpened opener</t>
+        </is>
+      </c>
+      <c r="J38" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2436,44 +2453,44 @@
           <t>cycling-active-recovery-explained</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C39" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D39" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E39" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F39" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G39" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H39" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion; genuinely x2</t>
+        </is>
+      </c>
+      <c r="I39" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY; stripped genuinely; tightened opener</t>
+        </is>
+      </c>
+      <c r="J39" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2486,44 +2503,44 @@
           <t>cycling-active-recovery-rides-guide</t>
         </is>
       </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G40" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H40" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I40" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J40" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C40" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E40" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F40" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G40" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="inlineStr">
+        <is>
+          <t>genuinely x6</t>
+        </is>
+      </c>
+      <c r="I40" s="28" t="inlineStr">
+        <is>
+          <t>Replaced 6 genuinely instances</t>
+        </is>
+      </c>
+      <c r="J40" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2536,44 +2553,44 @@
           <t>cycling-after-40-recovery-report-2026</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C41" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D41" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E41" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F41" s="28" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="G41" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H41" s="28" t="inlineStr">
+        <is>
+          <t>soft opener for stub format</t>
+        </is>
+      </c>
+      <c r="I41" s="28" t="inlineStr">
+        <is>
+          <t>Added em-dash contrast and fragment for sharper voice</t>
+        </is>
+      </c>
+      <c r="J41" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2586,44 +2603,44 @@
           <t>cycling-altitude-training</t>
         </is>
       </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G42" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I42" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J42" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C42" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E42" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F42" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G42" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="inlineStr">
+        <is>
+          <t>optimised x2; NDY expansion</t>
+        </is>
+      </c>
+      <c r="I42" s="28" t="inlineStr">
+        <is>
+          <t>Replaced optimised; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J42" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2636,44 +2653,44 @@
           <t>cycling-back-pain-fixes</t>
         </is>
       </c>
-      <c r="C43" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C43" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D43" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E43" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F43" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I43" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J43" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2686,44 +2703,44 @@
           <t>cycling-base-training-guide</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C44" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D44" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E44" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F44" s="28" t="inlineStr">
+        <is>
+          <t>9.7/10</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H44" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I44" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J44" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2736,44 +2753,44 @@
           <t>cycling-bike-upgrade-worth-it</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C45" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D45" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E45" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F45" s="28" t="inlineStr">
+        <is>
+          <t>9.6/10</t>
+        </is>
+      </c>
+      <c r="G45" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H45" s="28" t="inlineStr">
+        <is>
+          <t>transform your; optimise x3; NDY</t>
+        </is>
+      </c>
+      <c r="I45" s="28" t="inlineStr">
+        <is>
+          <t>Replaced transform your, optimise; expanded NDY</t>
+        </is>
+      </c>
+      <c r="J45" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2786,44 +2803,44 @@
           <t>cycling-body-composition-guide</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C46" s="27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E46" s="28" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+      <c r="F46" s="28" t="inlineStr">
+        <is>
+          <t>9.7/10</t>
+        </is>
+      </c>
+      <c r="G46" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H46" s="28" t="inlineStr">
+        <is>
+          <t>NDY expansion</t>
+        </is>
+      </c>
+      <c r="I46" s="28" t="inlineStr">
+        <is>
+          <t>Expanded NDY → Not Done Yet</t>
+        </is>
+      </c>
+      <c r="J46" s="28" t="inlineStr">
+        <is>
+          <t>Quality sweep 2026-05-08</t>
         </is>
       </c>
     </row>

</xml_diff>